<commit_message>
resolved the session refresh issue
</commit_message>
<xml_diff>
--- a/data/Batch_Products.xlsx
+++ b/data/Batch_Products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c84ab7d1c26c5bc5/Desktop/kiranwork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{50CADE15-27B4-4CEE-BCE0-A4C466A4B72D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8C93AEF-8858-473E-A038-08A88C1C94A7}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="8_{50CADE15-27B4-4CEE-BCE0-A4C466A4B72D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EB3F086-B850-4FC9-97BD-AE7742D5256F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E95B0DBA-EEC3-4033-92ED-3D487864D1C6}"/>
   </bookViews>
@@ -400,10 +400,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1471,9 +1467,15 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
+      <c r="L17" s="1">
+        <v>20</v>
+      </c>
+      <c r="M17" s="1">
+        <v>40</v>
+      </c>
+      <c r="N17" s="1">
+        <v>40</v>
+      </c>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
@@ -1511,9 +1513,15 @@
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
+      <c r="L18" s="1">
+        <v>50</v>
+      </c>
+      <c r="M18" s="1">
+        <v>10</v>
+      </c>
+      <c r="N18" s="1">
+        <v>40</v>
+      </c>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
@@ -1551,9 +1559,15 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
+      <c r="L19" s="1">
+        <v>10</v>
+      </c>
+      <c r="M19" s="1">
+        <v>20</v>
+      </c>
+      <c r="N19" s="1">
+        <v>70</v>
+      </c>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
@@ -1591,7 +1605,9 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
+      <c r="L20" s="1">
+        <v>10</v>
+      </c>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>

</xml_diff>